<commit_message>
Update dashboard — new photos and infrastructure data
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exports/mli1159_infrastructure29_04.xlsx
+++ b/exports/mli1159_infrastructure29_04.xlsx
@@ -5,22 +5,25 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Downloads\RMIS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Downloads\RMIS\RMIS_Dashboard\exports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F639588-C2E4-40DC-BA64-C358FB73E794}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD53E724-7B6E-4C76-AA0C-96AE52A27182}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cases" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Cases!$A$1:$AF$15</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="203">
   <si>
     <t>caseid</t>
   </si>
@@ -175,21 +178,12 @@
     <t>Réalisation de parc de vaccination Bangassi doudou-maure</t>
   </si>
   <si>
-    <t>9fcb6c12-3f93-47ec-be8a-544aee7f62d6</t>
-  </si>
-  <si>
     <t>urbaine_transfo_01</t>
   </si>
   <si>
     <t>autres_infrastructure</t>
   </si>
   <si>
-    <t>vidite site</t>
-  </si>
-  <si>
-    <t>13.0388726 -9.4735982 369.1 8.5</t>
-  </si>
-  <si>
     <t>2026-03-11</t>
   </si>
   <si>
@@ -197,21 +191,6 @@
   </si>
   <si>
     <t>Construction d’une unité de transformation multifonctionnellle à la commune urbaine de kita</t>
-  </si>
-  <si>
-    <t>site test</t>
-  </si>
-  <si>
-    <t>kolibougou</t>
-  </si>
-  <si>
-    <t>bienvenu.vuvalya</t>
-  </si>
-  <si>
-    <t>2026-03-11 10:29:28</t>
-  </si>
-  <si>
-    <t>https://eu.commcarehq.org/a/whh-mli/reports/case_data/9fcb6c12-3f93-47ec-be8a-544aee7f62d6/</t>
   </si>
   <si>
     <t>38c34e41-4787-498d-9f78-5f6b26762874</t>
@@ -1002,8 +981,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AF16"/>
+  <dimension ref="A1:AF15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="15" max="15" width="36.7109375" customWidth="1"/>
+    <col min="16" max="16" width="16.42578125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -1105,10 +1090,10 @@
     </row>
     <row r="2" spans="1:32" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B2" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="C2" t="s">
         <v>33</v>
@@ -1117,10 +1102,10 @@
         <v>33</v>
       </c>
       <c r="E2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F2" t="s">
         <v>53</v>
-      </c>
-      <c r="F2" t="s">
-        <v>33</v>
       </c>
       <c r="G2" t="s">
         <v>35</v>
@@ -1128,17 +1113,14 @@
       <c r="H2" t="s">
         <v>33</v>
       </c>
-      <c r="I2" t="s">
-        <v>54</v>
-      </c>
       <c r="J2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="K2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="L2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="M2" t="s">
         <v>33</v>
@@ -1147,10 +1129,10 @@
         <v>33</v>
       </c>
       <c r="O2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="P2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="Q2" t="s">
         <v>38</v>
@@ -1159,13 +1141,13 @@
         <v>33</v>
       </c>
       <c r="S2" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="T2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="U2" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="V2" t="s">
         <v>38</v>
@@ -1183,30 +1165,30 @@
         <v>33</v>
       </c>
       <c r="AA2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="AB2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="AC2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="AD2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="AE2" t="s">
         <v>40</v>
       </c>
       <c r="AF2" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:32" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="C3" t="s">
         <v>33</v>
@@ -1215,10 +1197,10 @@
         <v>33</v>
       </c>
       <c r="E3" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="F3" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="G3" t="s">
         <v>35</v>
@@ -1226,14 +1208,17 @@
       <c r="H3" t="s">
         <v>33</v>
       </c>
+      <c r="I3" t="s">
+        <v>69</v>
+      </c>
       <c r="J3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="K3" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="L3" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="M3" t="s">
         <v>33</v>
@@ -1242,10 +1227,10 @@
         <v>33</v>
       </c>
       <c r="O3" t="s">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="P3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q3" t="s">
         <v>38</v>
@@ -1254,13 +1239,13 @@
         <v>33</v>
       </c>
       <c r="S3" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="T3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="U3" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="V3" t="s">
         <v>38</v>
@@ -1278,30 +1263,30 @@
         <v>33</v>
       </c>
       <c r="AA3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="AB3" t="s">
+        <v>74</v>
+      </c>
+      <c r="AC3" t="s">
         <v>73</v>
       </c>
-      <c r="AC3" t="s">
-        <v>72</v>
-      </c>
       <c r="AD3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="AE3" t="s">
         <v>40</v>
       </c>
       <c r="AF3" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:32" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B4" t="s">
-        <v>52</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
         <v>33</v>
@@ -1310,7 +1295,7 @@
         <v>33</v>
       </c>
       <c r="E4" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="F4" t="s">
         <v>33</v>
@@ -1321,17 +1306,14 @@
       <c r="H4" t="s">
         <v>33</v>
       </c>
-      <c r="I4" t="s">
-        <v>77</v>
-      </c>
       <c r="J4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="K4" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="L4" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="M4" t="s">
         <v>33</v>
@@ -1340,10 +1322,10 @@
         <v>33</v>
       </c>
       <c r="O4" t="s">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="P4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="Q4" t="s">
         <v>38</v>
@@ -1352,13 +1334,13 @@
         <v>33</v>
       </c>
       <c r="S4" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="T4" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="U4" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="V4" t="s">
         <v>38</v>
@@ -1376,30 +1358,30 @@
         <v>33</v>
       </c>
       <c r="AA4" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="AB4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="AC4" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="AD4" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="AE4" t="s">
         <v>40</v>
       </c>
       <c r="AF4" s="1" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:32" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="B5" t="s">
-        <v>86</v>
+        <v>41</v>
       </c>
       <c r="C5" t="s">
         <v>33</v>
@@ -1408,7 +1390,7 @@
         <v>33</v>
       </c>
       <c r="E5" t="s">
-        <v>87</v>
+        <v>42</v>
       </c>
       <c r="F5" t="s">
         <v>33</v>
@@ -1420,13 +1402,13 @@
         <v>33</v>
       </c>
       <c r="J5" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="K5" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="L5" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="M5" t="s">
         <v>33</v>
@@ -1435,10 +1417,10 @@
         <v>33</v>
       </c>
       <c r="O5" t="s">
-        <v>90</v>
+        <v>44</v>
       </c>
       <c r="P5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="Q5" t="s">
         <v>38</v>
@@ -1450,10 +1432,10 @@
         <v>45</v>
       </c>
       <c r="T5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="U5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="V5" t="s">
         <v>38</v>
@@ -1471,13 +1453,13 @@
         <v>33</v>
       </c>
       <c r="AA5" t="s">
-        <v>93</v>
+        <v>64</v>
       </c>
       <c r="AB5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AC5" t="s">
-        <v>95</v>
+        <v>64</v>
       </c>
       <c r="AD5" t="s">
         <v>96</v>
@@ -1494,7 +1476,7 @@
         <v>98</v>
       </c>
       <c r="B6" t="s">
-        <v>41</v>
+        <v>99</v>
       </c>
       <c r="C6" t="s">
         <v>33</v>
@@ -1503,7 +1485,7 @@
         <v>33</v>
       </c>
       <c r="E6" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="F6" t="s">
         <v>33</v>
@@ -1515,13 +1497,13 @@
         <v>33</v>
       </c>
       <c r="J6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="K6" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="L6" t="s">
-        <v>43</v>
+        <v>101</v>
       </c>
       <c r="M6" t="s">
         <v>33</v>
@@ -1530,10 +1512,10 @@
         <v>33</v>
       </c>
       <c r="O6" t="s">
-        <v>44</v>
+        <v>102</v>
       </c>
       <c r="P6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="Q6" t="s">
         <v>38</v>
@@ -1545,7 +1527,7 @@
         <v>45</v>
       </c>
       <c r="T6" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="U6" t="s">
         <v>46</v>
@@ -1566,30 +1548,30 @@
         <v>33</v>
       </c>
       <c r="AA6" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="AB6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="AC6" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="AD6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="AE6" t="s">
         <v>40</v>
       </c>
       <c r="AF6" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" spans="1:32" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B7" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C7" t="s">
         <v>33</v>
@@ -1598,7 +1580,7 @@
         <v>33</v>
       </c>
       <c r="E7" t="s">
-        <v>34</v>
+        <v>79</v>
       </c>
       <c r="F7" t="s">
         <v>33</v>
@@ -1609,14 +1591,17 @@
       <c r="H7" t="s">
         <v>33</v>
       </c>
+      <c r="I7" t="s">
+        <v>110</v>
+      </c>
       <c r="J7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="K7" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="L7" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="M7" t="s">
         <v>33</v>
@@ -1625,10 +1610,10 @@
         <v>33</v>
       </c>
       <c r="O7" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="P7" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="Q7" t="s">
         <v>38</v>
@@ -1640,7 +1625,7 @@
         <v>45</v>
       </c>
       <c r="T7" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="U7" t="s">
         <v>46</v>
@@ -1661,30 +1646,30 @@
         <v>33</v>
       </c>
       <c r="AA7" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="AB7" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="AC7" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="AD7" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AE7" t="s">
         <v>40</v>
       </c>
       <c r="AF7" s="1" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="8" spans="1:32" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B8" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C8" t="s">
         <v>33</v>
@@ -1693,7 +1678,7 @@
         <v>33</v>
       </c>
       <c r="E8" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="F8" t="s">
         <v>33</v>
@@ -1705,16 +1690,16 @@
         <v>33</v>
       </c>
       <c r="I8" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="J8" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="K8" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="L8" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="M8" t="s">
         <v>33</v>
@@ -1723,10 +1708,10 @@
         <v>33</v>
       </c>
       <c r="O8" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="P8" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="Q8" t="s">
         <v>38</v>
@@ -1738,10 +1723,10 @@
         <v>45</v>
       </c>
       <c r="T8" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="U8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="V8" t="s">
         <v>38</v>
@@ -1759,30 +1744,30 @@
         <v>33</v>
       </c>
       <c r="AA8" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="AB8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="AC8" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="AD8" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="AE8" t="s">
         <v>40</v>
       </c>
       <c r="AF8" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:32" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B9" t="s">
-        <v>128</v>
+        <v>47</v>
       </c>
       <c r="C9" t="s">
         <v>33</v>
@@ -1791,7 +1776,7 @@
         <v>33</v>
       </c>
       <c r="E9" t="s">
-        <v>87</v>
+        <v>48</v>
       </c>
       <c r="F9" t="s">
         <v>33</v>
@@ -1802,17 +1787,14 @@
       <c r="H9" t="s">
         <v>33</v>
       </c>
-      <c r="I9" t="s">
-        <v>129</v>
-      </c>
       <c r="J9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K9" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="L9" t="s">
-        <v>131</v>
+        <v>49</v>
       </c>
       <c r="M9" t="s">
         <v>33</v>
@@ -1821,7 +1803,7 @@
         <v>33</v>
       </c>
       <c r="O9" t="s">
-        <v>132</v>
+        <v>50</v>
       </c>
       <c r="P9" t="s">
         <v>133</v>
@@ -1857,13 +1839,13 @@
         <v>33</v>
       </c>
       <c r="AA9" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="AB9" t="s">
         <v>135</v>
       </c>
       <c r="AC9" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="AD9" t="s">
         <v>136</v>
@@ -1880,7 +1862,7 @@
         <v>138</v>
       </c>
       <c r="B10" t="s">
-        <v>47</v>
+        <v>139</v>
       </c>
       <c r="C10" t="s">
         <v>33</v>
@@ -1889,7 +1871,7 @@
         <v>33</v>
       </c>
       <c r="E10" t="s">
-        <v>48</v>
+        <v>140</v>
       </c>
       <c r="F10" t="s">
         <v>33</v>
@@ -1901,13 +1883,13 @@
         <v>33</v>
       </c>
       <c r="J10" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="K10" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="L10" t="s">
-        <v>49</v>
+        <v>143</v>
       </c>
       <c r="M10" t="s">
         <v>33</v>
@@ -1916,10 +1898,10 @@
         <v>33</v>
       </c>
       <c r="O10" t="s">
-        <v>50</v>
+        <v>144</v>
       </c>
       <c r="P10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="Q10" t="s">
         <v>38</v>
@@ -1928,13 +1910,13 @@
         <v>33</v>
       </c>
       <c r="S10" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="T10" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="U10" t="s">
-        <v>45</v>
+        <v>147</v>
       </c>
       <c r="V10" t="s">
         <v>38</v>
@@ -1952,30 +1934,30 @@
         <v>33</v>
       </c>
       <c r="AA10" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="AB10" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="AC10" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="AD10" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="AE10" t="s">
         <v>40</v>
       </c>
       <c r="AF10" s="1" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11" spans="1:32" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="B11" t="s">
-        <v>147</v>
+        <v>32</v>
       </c>
       <c r="C11" t="s">
         <v>33</v>
@@ -1984,7 +1966,7 @@
         <v>33</v>
       </c>
       <c r="E11" t="s">
-        <v>148</v>
+        <v>34</v>
       </c>
       <c r="F11" t="s">
         <v>33</v>
@@ -1996,13 +1978,13 @@
         <v>33</v>
       </c>
       <c r="J11" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="K11" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="L11" t="s">
-        <v>151</v>
+        <v>36</v>
       </c>
       <c r="M11" t="s">
         <v>33</v>
@@ -2011,7 +1993,7 @@
         <v>33</v>
       </c>
       <c r="O11" t="s">
-        <v>152</v>
+        <v>37</v>
       </c>
       <c r="P11" t="s">
         <v>153</v>
@@ -2029,7 +2011,7 @@
         <v>154</v>
       </c>
       <c r="U11" t="s">
-        <v>155</v>
+        <v>39</v>
       </c>
       <c r="V11" t="s">
         <v>38</v>
@@ -2047,13 +2029,13 @@
         <v>33</v>
       </c>
       <c r="AA11" t="s">
-        <v>93</v>
+        <v>155</v>
       </c>
       <c r="AB11" t="s">
         <v>156</v>
       </c>
       <c r="AC11" t="s">
-        <v>93</v>
+        <v>155</v>
       </c>
       <c r="AD11" t="s">
         <v>157</v>
@@ -2070,7 +2052,7 @@
         <v>159</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>160</v>
       </c>
       <c r="C12" t="s">
         <v>33</v>
@@ -2079,7 +2061,7 @@
         <v>33</v>
       </c>
       <c r="E12" t="s">
-        <v>34</v>
+        <v>79</v>
       </c>
       <c r="F12" t="s">
         <v>33</v>
@@ -2090,14 +2072,17 @@
       <c r="H12" t="s">
         <v>33</v>
       </c>
+      <c r="I12" t="s">
+        <v>161</v>
+      </c>
       <c r="J12" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="K12" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="L12" t="s">
-        <v>36</v>
+        <v>164</v>
       </c>
       <c r="M12" t="s">
         <v>33</v>
@@ -2106,10 +2091,10 @@
         <v>33</v>
       </c>
       <c r="O12" t="s">
-        <v>37</v>
+        <v>165</v>
       </c>
       <c r="P12" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="Q12" t="s">
         <v>38</v>
@@ -2121,7 +2106,7 @@
         <v>39</v>
       </c>
       <c r="T12" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="U12" t="s">
         <v>39</v>
@@ -2142,30 +2127,30 @@
         <v>33</v>
       </c>
       <c r="AA12" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="AB12" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="AC12" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="AD12" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="AE12" t="s">
         <v>40</v>
       </c>
       <c r="AF12" s="1" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
     </row>
     <row r="13" spans="1:32" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="B13" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="C13" t="s">
         <v>33</v>
@@ -2174,7 +2159,7 @@
         <v>33</v>
       </c>
       <c r="E13" t="s">
-        <v>87</v>
+        <v>34</v>
       </c>
       <c r="F13" t="s">
         <v>33</v>
@@ -2185,17 +2170,14 @@
       <c r="H13" t="s">
         <v>33</v>
       </c>
-      <c r="I13" t="s">
-        <v>169</v>
-      </c>
       <c r="J13" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="K13" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="L13" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="M13" t="s">
         <v>33</v>
@@ -2204,10 +2186,10 @@
         <v>33</v>
       </c>
       <c r="O13" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="P13" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="Q13" t="s">
         <v>38</v>
@@ -2219,7 +2201,7 @@
         <v>39</v>
       </c>
       <c r="T13" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="U13" t="s">
         <v>39</v>
@@ -2240,30 +2222,30 @@
         <v>33</v>
       </c>
       <c r="AA13" t="s">
-        <v>176</v>
+        <v>155</v>
       </c>
       <c r="AB13" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="AC13" t="s">
-        <v>176</v>
+        <v>155</v>
       </c>
       <c r="AD13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="AE13" t="s">
         <v>40</v>
       </c>
       <c r="AF13" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="14" spans="1:32" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B14" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C14" t="s">
         <v>33</v>
@@ -2272,7 +2254,7 @@
         <v>33</v>
       </c>
       <c r="E14" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="F14" t="s">
         <v>33</v>
@@ -2283,14 +2265,17 @@
       <c r="H14" t="s">
         <v>33</v>
       </c>
+      <c r="I14" t="s">
+        <v>183</v>
+      </c>
       <c r="J14" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="K14" t="s">
-        <v>171</v>
+        <v>185</v>
       </c>
       <c r="L14" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
       <c r="M14" t="s">
         <v>33</v>
@@ -2299,10 +2284,10 @@
         <v>33</v>
       </c>
       <c r="O14" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="P14" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="Q14" t="s">
         <v>38</v>
@@ -2314,10 +2299,10 @@
         <v>39</v>
       </c>
       <c r="T14" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="U14" t="s">
-        <v>39</v>
+        <v>186</v>
       </c>
       <c r="V14" t="s">
         <v>38</v>
@@ -2335,30 +2320,30 @@
         <v>33</v>
       </c>
       <c r="AA14" t="s">
-        <v>163</v>
+        <v>190</v>
       </c>
       <c r="AB14" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="AC14" t="s">
-        <v>163</v>
+        <v>190</v>
       </c>
       <c r="AD14" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="AE14" t="s">
         <v>40</v>
       </c>
       <c r="AF14" s="1" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
     </row>
     <row r="15" spans="1:32" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="B15" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="C15" t="s">
         <v>33</v>
@@ -2367,7 +2352,7 @@
         <v>33</v>
       </c>
       <c r="E15" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="F15" t="s">
         <v>33</v>
@@ -2379,16 +2364,16 @@
         <v>33</v>
       </c>
       <c r="I15" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="J15" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="K15" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="L15" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="M15" t="s">
         <v>33</v>
@@ -2397,10 +2382,10 @@
         <v>33</v>
       </c>
       <c r="O15" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="P15" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="Q15" t="s">
         <v>38</v>
@@ -2412,10 +2397,10 @@
         <v>39</v>
       </c>
       <c r="T15" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
       <c r="U15" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="V15" t="s">
         <v>38</v>
@@ -2433,139 +2418,40 @@
         <v>33</v>
       </c>
       <c r="AA15" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="AB15" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="AC15" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="AD15" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="AE15" t="s">
         <v>40</v>
       </c>
       <c r="AF15" s="1" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="16" spans="1:32" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
         <v>202</v>
-      </c>
-      <c r="B16" t="s">
-        <v>203</v>
-      </c>
-      <c r="C16" t="s">
-        <v>33</v>
-      </c>
-      <c r="D16" t="s">
-        <v>33</v>
-      </c>
-      <c r="E16" t="s">
-        <v>53</v>
-      </c>
-      <c r="F16" t="s">
-        <v>33</v>
-      </c>
-      <c r="G16" t="s">
-        <v>35</v>
-      </c>
-      <c r="H16" t="s">
-        <v>33</v>
-      </c>
-      <c r="I16" t="s">
-        <v>204</v>
-      </c>
-      <c r="J16" t="s">
-        <v>205</v>
-      </c>
-      <c r="K16" t="s">
-        <v>193</v>
-      </c>
-      <c r="L16" t="s">
-        <v>194</v>
-      </c>
-      <c r="M16" t="s">
-        <v>33</v>
-      </c>
-      <c r="N16" t="s">
-        <v>33</v>
-      </c>
-      <c r="O16" t="s">
-        <v>206</v>
-      </c>
-      <c r="P16" t="s">
-        <v>207</v>
-      </c>
-      <c r="Q16" t="s">
-        <v>38</v>
-      </c>
-      <c r="R16" t="s">
-        <v>33</v>
-      </c>
-      <c r="S16" t="s">
-        <v>39</v>
-      </c>
-      <c r="T16" t="s">
-        <v>194</v>
-      </c>
-      <c r="U16" t="s">
-        <v>194</v>
-      </c>
-      <c r="V16" t="s">
-        <v>38</v>
-      </c>
-      <c r="W16" t="s">
-        <v>38</v>
-      </c>
-      <c r="X16" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y16" t="s">
-        <v>33</v>
-      </c>
-      <c r="Z16" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA16" t="s">
-        <v>198</v>
-      </c>
-      <c r="AB16" t="s">
-        <v>208</v>
-      </c>
-      <c r="AC16" t="s">
-        <v>198</v>
-      </c>
-      <c r="AD16" t="s">
-        <v>209</v>
-      </c>
-      <c r="AE16" t="s">
-        <v>40</v>
-      </c>
-      <c r="AF16" s="1" t="s">
-        <v>210</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="AF2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="AF3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="AF4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="AF5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="AF6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="AF7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="AF8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="AF9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="AF10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="AF11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="AF12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="AF13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="AF14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="AF15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="AF16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="AF2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="AF3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="AF4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="AF5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="AF6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="AF7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="AF8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="AF9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="AF10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="AF11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="AF12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="AF13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="AF14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="AF15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>